<commit_message>
Update negative price analysis 2026-04
</commit_message>
<xml_diff>
--- a/outputs/All_States_negative_prices.xlsx
+++ b/outputs/All_States_negative_prices.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NSW" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QLD" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VIC" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SA" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TAS" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="NSW" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="QLD" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="VIC" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="SA" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="TAS" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
Update negative price analysis 2026-05
</commit_message>
<xml_diff>
--- a/outputs/All_States_negative_prices.xlsx
+++ b/outputs/All_States_negative_prices.xlsx
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J84"/>
+  <dimension ref="A1:J85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3333,6 +3333,40 @@
         <v>0</v>
       </c>
     </row>
+    <row r="85">
+      <c r="A85" s="2" t="inlineStr">
+        <is>
+          <t>Apr 2026</t>
+        </is>
+      </c>
+      <c r="B85" s="3" t="n">
+        <v>19.2</v>
+      </c>
+      <c r="C85" s="3" t="n">
+        <v>2.15</v>
+      </c>
+      <c r="D85" s="3" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="E85" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F85" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G85" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H85" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I85" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J85" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3344,7 +3378,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J84"/>
+  <dimension ref="A1:J85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6233,6 +6267,40 @@
         <v>0</v>
       </c>
     </row>
+    <row r="85">
+      <c r="A85" s="2" t="inlineStr">
+        <is>
+          <t>Apr 2026</t>
+        </is>
+      </c>
+      <c r="B85" s="3" t="n">
+        <v>39.06</v>
+      </c>
+      <c r="C85" s="3" t="n">
+        <v>1.98</v>
+      </c>
+      <c r="D85" s="3" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="E85" s="3" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="F85" s="3" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="G85" s="3" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="H85" s="3" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="I85" s="3" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="J85" s="3" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -6244,7 +6312,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J84"/>
+  <dimension ref="A1:J85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -9133,6 +9201,40 @@
         <v>0.03</v>
       </c>
     </row>
+    <row r="85">
+      <c r="A85" s="2" t="inlineStr">
+        <is>
+          <t>Apr 2026</t>
+        </is>
+      </c>
+      <c r="B85" s="3" t="n">
+        <v>56.49</v>
+      </c>
+      <c r="C85" s="3" t="n">
+        <v>21.25</v>
+      </c>
+      <c r="D85" s="3" t="n">
+        <v>10.24</v>
+      </c>
+      <c r="E85" s="3" t="n">
+        <v>7.81</v>
+      </c>
+      <c r="F85" s="3" t="n">
+        <v>5.97</v>
+      </c>
+      <c r="G85" s="3" t="n">
+        <v>4.62</v>
+      </c>
+      <c r="H85" s="3" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="I85" s="3" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="J85" s="3" t="n">
+        <v>0.35</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -9144,7 +9246,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J84"/>
+  <dimension ref="A1:J85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -12033,6 +12135,40 @@
         <v>11.53</v>
       </c>
     </row>
+    <row r="85">
+      <c r="A85" s="2" t="inlineStr">
+        <is>
+          <t>Apr 2026</t>
+        </is>
+      </c>
+      <c r="B85" s="3" t="n">
+        <v>54.17</v>
+      </c>
+      <c r="C85" s="3" t="n">
+        <v>18.23</v>
+      </c>
+      <c r="D85" s="3" t="n">
+        <v>6.98</v>
+      </c>
+      <c r="E85" s="3" t="n">
+        <v>6.18</v>
+      </c>
+      <c r="F85" s="3" t="n">
+        <v>5.66</v>
+      </c>
+      <c r="G85" s="3" t="n">
+        <v>4.62</v>
+      </c>
+      <c r="H85" s="3" t="n">
+        <v>2.64</v>
+      </c>
+      <c r="I85" s="3" t="n">
+        <v>1.63</v>
+      </c>
+      <c r="J85" s="3" t="n">
+        <v>1.46</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -12044,7 +12180,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J84"/>
+  <dimension ref="A1:J85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -14933,6 +15069,40 @@
         <v>0</v>
       </c>
     </row>
+    <row r="85">
+      <c r="A85" s="2" t="inlineStr">
+        <is>
+          <t>Apr 2026</t>
+        </is>
+      </c>
+      <c r="B85" s="3" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="C85" s="3" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="D85" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E85" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F85" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G85" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H85" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I85" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J85" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update negative price analysis 2026-07
</commit_message>
<xml_diff>
--- a/outputs/All_States_negative_prices.xlsx
+++ b/outputs/All_States_negative_prices.xlsx
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J85"/>
+  <dimension ref="A1:J86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3367,6 +3367,40 @@
         <v>0</v>
       </c>
     </row>
+    <row r="86">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="B86" s="3" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="C86" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D86" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E86" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F86" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G86" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H86" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I86" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J86" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3378,7 +3412,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J85"/>
+  <dimension ref="A1:J86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6301,6 +6335,40 @@
         <v>0.07000000000000001</v>
       </c>
     </row>
+    <row r="86">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="B86" s="3" t="n">
+        <v>18.65</v>
+      </c>
+      <c r="C86" s="3" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="D86" s="3" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="E86" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F86" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G86" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H86" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I86" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J86" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -6312,7 +6380,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J85"/>
+  <dimension ref="A1:J86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -9235,6 +9303,40 @@
         <v>0.35</v>
       </c>
     </row>
+    <row r="86">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="B86" s="3" t="n">
+        <v>21.64</v>
+      </c>
+      <c r="C86" s="3" t="n">
+        <v>1.04</v>
+      </c>
+      <c r="D86" s="3" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="E86" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F86" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G86" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H86" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I86" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J86" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -9246,7 +9348,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J85"/>
+  <dimension ref="A1:J86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -12169,6 +12271,40 @@
         <v>1.46</v>
       </c>
     </row>
+    <row r="86">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="B86" s="3" t="n">
+        <v>18.51</v>
+      </c>
+      <c r="C86" s="3" t="n">
+        <v>0.47</v>
+      </c>
+      <c r="D86" s="3" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="E86" s="3" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="F86" s="3" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="G86" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H86" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I86" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J86" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -12180,7 +12316,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J85"/>
+  <dimension ref="A1:J86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -15103,6 +15239,40 @@
         <v>0</v>
       </c>
     </row>
+    <row r="86">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="B86" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C86" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D86" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E86" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F86" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G86" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H86" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I86" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J86" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update negative price analysis 2026-10
</commit_message>
<xml_diff>
--- a/outputs/All_States_negative_prices.xlsx
+++ b/outputs/All_States_negative_prices.xlsx
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J88"/>
+  <dimension ref="A1:J89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3469,6 +3469,40 @@
         <v>0</v>
       </c>
     </row>
+    <row r="89">
+      <c r="A89" s="2" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="B89" s="3" t="n">
+        <v>6.92</v>
+      </c>
+      <c r="C89" s="3" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="D89" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E89" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F89" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G89" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H89" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I89" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J89" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3480,7 +3514,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J88"/>
+  <dimension ref="A1:J89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6505,6 +6539,40 @@
         <v>0</v>
       </c>
     </row>
+    <row r="89">
+      <c r="A89" s="2" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="B89" s="3" t="n">
+        <v>34.27</v>
+      </c>
+      <c r="C89" s="3" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="D89" s="3" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E89" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F89" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G89" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H89" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I89" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J89" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -6516,7 +6584,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J88"/>
+  <dimension ref="A1:J89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -9541,6 +9609,40 @@
         <v>0.27</v>
       </c>
     </row>
+    <row r="89">
+      <c r="A89" s="2" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="B89" s="3" t="n">
+        <v>22.55</v>
+      </c>
+      <c r="C89" s="3" t="n">
+        <v>3.26</v>
+      </c>
+      <c r="D89" s="3" t="n">
+        <v>1.31</v>
+      </c>
+      <c r="E89" s="3" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="F89" s="3" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="G89" s="3" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="H89" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I89" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J89" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -9552,7 +9654,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J88"/>
+  <dimension ref="A1:J89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -12577,6 +12679,40 @@
         <v>0.44</v>
       </c>
     </row>
+    <row r="89">
+      <c r="A89" s="2" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="B89" s="3" t="n">
+        <v>29.23</v>
+      </c>
+      <c r="C89" s="3" t="n">
+        <v>4.77</v>
+      </c>
+      <c r="D89" s="3" t="n">
+        <v>1.88</v>
+      </c>
+      <c r="E89" s="3" t="n">
+        <v>1.68</v>
+      </c>
+      <c r="F89" s="3" t="n">
+        <v>1.34</v>
+      </c>
+      <c r="G89" s="3" t="n">
+        <v>1.18</v>
+      </c>
+      <c r="H89" s="3" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="I89" s="3" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="J89" s="3" t="n">
+        <v>0.74</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -12588,7 +12724,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J88"/>
+  <dimension ref="A1:J89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -15613,6 +15749,40 @@
         <v>0</v>
       </c>
     </row>
+    <row r="89">
+      <c r="A89" s="2" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="B89" s="3" t="n">
+        <v>18.18</v>
+      </c>
+      <c r="C89" s="3" t="n">
+        <v>2.22</v>
+      </c>
+      <c r="D89" s="3" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="E89" s="3" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="F89" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G89" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H89" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I89" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J89" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Regenerate workbooks: one fixed heat scale and a % unit (summary.csv unchanged)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/All_States_negative_prices.xlsx
+++ b/outputs/All_States_negative_prices.xlsx
@@ -20,7 +20,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.00&quot;%&quot;"/>
+  </numFmts>
   <fonts count="3">
     <font>
       <name val="Calibri"/>
@@ -76,7 +78,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>

</xml_diff>